<commit_message>
Change EXTRA packets to INFO - not validated but acceptable
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
+++ b/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
@@ -92,16 +92,16 @@
     <x:t>Enter operation (format as A X B):</x:t>
   </x:si>
   <x:si>
-    <x:t>PASS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NONE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>None</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Text comparison passed: client output matches exactly</x:t>
+    <x:t>FAIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>COMPARE_FAIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OutputMismatch</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Text comparison failed: client output mismatch</x:t>
   </x:si>
   <x:si>
     <x:t>ServerStdout</x:t>
@@ -110,30 +110,9 @@
     <x:t>Waiting for a connection from client</x:t>
   </x:si>
   <x:si>
-    <x:t>FAIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>COMPARE_FAIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OutputMismatch</x:t>
-  </x:si>
-  <x:si>
     <x:t>Text comparison failed: server output mismatch</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">The command could not be loaded, possibly because:
-  * You intended to execute a .NET application:
-      The application '/apps/Server/Project11.dll' does not exist.
-  * You intended to execute a .NET SDK command:
-      No .NET SDKs were found.
-Download a .NET SDK:
-https://aka.ms/dotnet/download
-Learn about SDK resolution:
-https://aka.ms/dotnet/sdk-not-found
-</x:t>
-  </x:si>
-  <x:si>
     <x:t>Time</x:t>
   </x:si>
   <x:si>
@@ -194,6 +173,9 @@
     <x:t>Server</x:t>
   </x:si>
   <x:si>
+    <x:t>(MISSING - not captured)</x:t>
+  </x:si>
+  <x:si>
     <x:t>SYN, ACK</x:t>
   </x:si>
   <x:si>
@@ -210,28 +192,6 @@
   </x:si>
   <x:si>
     <x:t>Data transfer in progress</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACK, PSH</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1 + 2
-</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PARTIAL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(EXTRA - not expected)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EXTRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ACK, RST</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Connection reset (RST) - Error occurred</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -258,7 +218,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -267,17 +227,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF90EE90"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFF00"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFE0"/>
+        <x:fgColor rgb="FFFFB6C1"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -300,7 +250,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="5">
+  <x:cellStyleXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -310,14 +260,8 @@
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -326,19 +270,7 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -766,19 +698,19 @@
     <x:col min="4" max="4" width="9.424911" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.424911" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.282054" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13.567768" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14.996339" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16.424911" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="14.567768" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="13.996339" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="11.567768" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="10.139196" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="50.139196" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="43.282054" style="0" customWidth="1"/>
     <x:col min="14" max="14" width="8.853482" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="15.567768" style="0" customWidth="1"/>
     <x:col min="16" max="16" width="13.139196" style="0" customWidth="1"/>
     <x:col min="17" max="17" width="15.567768" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="13.139196" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="30.853482" style="0" customWidth="1"/>
+    <x:col min="19" max="19" width="11.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:19" s="1" customFormat="1">
@@ -869,7 +801,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="S2" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -907,7 +839,7 @@
     <x:col min="16" max="16" width="13.139196" style="0" customWidth="1"/>
     <x:col min="17" max="17" width="15.567768" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="13.139196" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="56.424911" style="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12.853482" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:19" s="1" customFormat="1">
@@ -977,13 +909,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="I2" s="0">
         <x:v>0</x:v>
@@ -995,10 +927,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="S2" s="2" t="s">
-        <x:v>34</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="S2" s="0" t="s">
+        <x:v>17</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1031,11 +963,11 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:P9"/>
+  <x:dimension ref="A1:P6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="5.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="5.139196" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="4.424911" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="6.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="11.139196" style="0" customWidth="1"/>
@@ -1044,8 +976,8 @@
     <x:col min="8" max="8" width="4.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="15.139196" style="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10.853482" style="0" customWidth="1"/>
-    <x:col min="12" max="12" width="35.710625" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.424911" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="10.996339" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="16.424911" style="0" customWidth="1"/>
     <x:col min="14" max="14" width="14.424911" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="10.567768" style="0" customWidth="1"/>
@@ -1057,49 +989,49 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="C1" s="1" t="s">
+      <x:c r="G1" s="1" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="D1" s="1" t="s">
+      <x:c r="H1" s="1" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="E1" s="1" t="s">
+      <x:c r="I1" s="1" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="s">
+      <x:c r="J1" s="1" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="G1" s="1" t="s">
+      <x:c r="K1" s="1" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="H1" s="1" t="s">
+      <x:c r="L1" s="1" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="I1" s="1" t="s">
+      <x:c r="M1" s="1" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="J1" s="1" t="s">
+      <x:c r="N1" s="1" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="K1" s="1" t="s">
+      <x:c r="O1" s="1" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="L1" s="1" t="s">
+      <x:c r="P1" s="1" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="M1" s="1" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="N1" s="1" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="O1" s="1" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="P1" s="1" t="s">
-        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:16">
@@ -1110,45 +1042,45 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F2" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="H2" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I2" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="J2" s="0" t="s">
-        <x:v>54</x:v>
       </x:c>
       <x:c r="K2" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="O2" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P2" s="3" t="s">
+      <x:c r="P2" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1160,45 +1092,45 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="J3" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="K3" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N3" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="O3" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P3" s="3" t="s">
+      <x:c r="P3" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1210,45 +1142,45 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I4" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="K4" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N4" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="O4" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P4" s="3" t="s">
+      <x:c r="P4" s="2" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1260,46 +1192,46 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J5" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F5" s="0" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G5" s="0" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="H5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I5" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="J5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="K5" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L5" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M5" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O5" s="2" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="P5" s="4" t="s">
-        <x:v>63</x:v>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="O5" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="P5" s="2" t="s">
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:16">
@@ -1310,196 +1242,46 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="G6" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="H6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I6" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
       <x:c r="J6" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="K6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L6" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M6" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N6" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="O6" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P6" s="3" t="s">
+      <x:c r="P6" s="2" t="s">
         <x:v>24</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:16">
-      <x:c r="A7" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="J7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K7" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="L7" s="0" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="M7" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="N7" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="O7" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P7" s="5" t="s">
-        <x:v>65</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:16">
-      <x:c r="A8" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="J8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K8" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="L8" s="0" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="M8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="N8" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="O8" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P8" s="5" t="s">
-        <x:v>65</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:16">
-      <x:c r="A9" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="J9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K9" s="0" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="L9" s="0" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="M9" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="N9" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="O9" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P9" s="5" t="s">
-        <x:v>65</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Complete parallel grading test: 3 students, batches of 2, all requirements verified
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
+++ b/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
@@ -92,6 +92,24 @@
     <x:t>Enter operation (format as A X B):</x:t>
   </x:si>
   <x:si>
+    <x:t>PASS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NONE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>None</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Text comparison passed: client output matches exactly</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ServerStdout</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Waiting for a connection from client</x:t>
+  </x:si>
+  <x:si>
     <x:t>FAIL</x:t>
   </x:si>
   <x:si>
@@ -101,18 +119,21 @@
     <x:t>OutputMismatch</x:t>
   </x:si>
   <x:si>
-    <x:t>Text comparison failed: client output mismatch</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ServerStdout</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Waiting for a connection from client</x:t>
-  </x:si>
-  <x:si>
     <x:t>Text comparison failed: server output mismatch</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">The command could not be loaded, possibly because:
+  * You intended to execute a .NET application:
+      The application '/apps/Server/Project11.dll' does not exist.
+  * You intended to execute a .NET SDK command:
+      No .NET SDKs were found.
+Download a .NET SDK:
+https://aka.ms/dotnet/download
+Learn about SDK resolution:
+https://aka.ms/dotnet/sdk-not-found
+</x:t>
+  </x:si>
+  <x:si>
     <x:t>Time</x:t>
   </x:si>
   <x:si>
@@ -173,9 +194,6 @@
     <x:t>Server</x:t>
   </x:si>
   <x:si>
-    <x:t>(MISSING - not captured)</x:t>
-  </x:si>
-  <x:si>
     <x:t>SYN, ACK</x:t>
   </x:si>
   <x:si>
@@ -192,6 +210,28 @@
   </x:si>
   <x:si>
     <x:t>Data transfer in progress</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACK, PSH</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">1 + 2
+</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PARTIAL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACK, RST</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Connection reset (RST) - Error occurred</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(Not validated by this test case)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INFO</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -218,7 +258,7 @@
       <x:family val="2"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -227,7 +267,17 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFB6C1"/>
+        <x:fgColor rgb="FF90EE90"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFF00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD3D3D3"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -250,7 +300,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="3">
+  <x:cellStyleXfs count="5">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -260,8 +310,14 @@
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -270,7 +326,19 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -698,19 +766,19 @@
     <x:col min="4" max="4" width="9.424911" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="6.424911" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="6.282054" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14.996339" style="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13.567768" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="14.567768" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="13.996339" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="11.567768" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="10.139196" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="43.282054" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="50.139196" style="0" customWidth="1"/>
     <x:col min="14" max="14" width="8.853482" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="15.567768" style="0" customWidth="1"/>
     <x:col min="16" max="16" width="13.139196" style="0" customWidth="1"/>
     <x:col min="17" max="17" width="15.567768" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="13.139196" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="11.996339" style="0" customWidth="1"/>
+    <x:col min="19" max="19" width="30.853482" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:19" s="1" customFormat="1">
@@ -801,7 +869,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="S2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -839,7 +907,7 @@
     <x:col min="16" max="16" width="13.139196" style="0" customWidth="1"/>
     <x:col min="17" max="17" width="15.567768" style="0" customWidth="1"/>
     <x:col min="18" max="18" width="13.139196" style="0" customWidth="1"/>
-    <x:col min="19" max="19" width="12.853482" style="0" customWidth="1"/>
+    <x:col min="19" max="19" width="56.424911" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:19" s="1" customFormat="1">
@@ -909,13 +977,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="I2" s="0">
         <x:v>0</x:v>
@@ -927,10 +995,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="S2" s="2" t="s">
+        <x:v>34</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -963,11 +1031,11 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:P6"/>
+  <x:dimension ref="A1:P9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="5.710625" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="5.139196" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="4.424911" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="6.853482" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="11.139196" style="0" customWidth="1"/>
@@ -976,8 +1044,8 @@
     <x:col min="8" max="8" width="4.996339" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="10.853482" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="15.139196" style="0" customWidth="1"/>
-    <x:col min="11" max="11" width="23.424911" style="0" customWidth="1"/>
-    <x:col min="12" max="12" width="10.996339" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="10.853482" style="0" customWidth="1"/>
+    <x:col min="12" max="12" width="35.710625" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="16.424911" style="0" customWidth="1"/>
     <x:col min="14" max="14" width="14.424911" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="10.567768" style="0" customWidth="1"/>
@@ -989,49 +1057,49 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>32</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="I1" s="1" t="s">
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="J1" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="K1" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="L1" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="M1" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="N1" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="O1" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="P1" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:16">
@@ -1042,7 +1110,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>17</x:v>
@@ -1051,36 +1119,36 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K2" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="N2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="O2" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P2" s="2" t="s">
+      <x:c r="P2" s="3" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1092,7 +1160,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
         <x:v>17</x:v>
@@ -1101,36 +1169,36 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I3" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
       <x:c r="K3" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="N3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="O3" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P3" s="2" t="s">
+      <x:c r="P3" s="3" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1142,7 +1210,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
         <x:v>17</x:v>
@@ -1151,36 +1219,36 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I4" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="J4" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="K4" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="N4" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="O4" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="P4" s="2" t="s">
+      <x:c r="P4" s="3" t="s">
         <x:v>24</x:v>
       </x:c>
     </x:row>
@@ -1192,7 +1260,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
         <x:v>17</x:v>
@@ -1201,37 +1269,37 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H5" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="J5" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="K5" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="L5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="M5" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="N5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="O5" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P5" s="2" t="s">
-        <x:v>24</x:v>
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="O5" s="2" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="P5" s="4" t="s">
+        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:16">
@@ -1242,7 +1310,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
         <x:v>17</x:v>
@@ -1251,37 +1319,187 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I6" s="0" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="G6" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="H6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="I6" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="J6" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="K6" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="L6" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="M6" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="N6" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="O6" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="P6" s="4" t="s">
+        <x:v>63</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:16">
+      <x:c r="A7" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K7" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="L6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="M6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="N6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="O6" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="P6" s="2" t="s">
-        <x:v>24</x:v>
+      <x:c r="L7" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M7" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="N7" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="O7" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="P7" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:16">
+      <x:c r="A8" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K8" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="L8" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="M8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="N8" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="O8" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="P8" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:16">
+      <x:c r="A9" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="J9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K9" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="L9" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="M9" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="N9" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="O9" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="P9" s="5" t="s">
+        <x:v>67</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Final test - Docker images rebuilt, all fixes verified working
Co-authored-by: NguyenHuuCuongK18 <169327600+NguyenHuuCuongK18@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
+++ b/Submit/Results/cuongnhhe186494/TC2_Send/GradeDetail.xlsx
@@ -212,6 +212,15 @@
   </x:si>
   <x:si>
     <x:t>INFO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ACK, FIN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Closing connection (FIN-ACK)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RST</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1402,10 +1411,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="K8" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="L8" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M8" s="0" t="s">
         <x:v>51</x:v>
@@ -1452,7 +1461,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="K9" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="L9" s="0" t="s">
         <x:v>61</x:v>

</xml_diff>